<commit_message>
Guide: row insertion, dropdown and Protected View notes, --capacity, new checks; regenerate workbook
</commit_message>
<xml_diff>
--- a/docs/crane-statics-validation-22689.xlsx
+++ b/docs/crane-statics-validation-22689.xlsx
@@ -7002,52 +7002,52 @@
     </row>
   </sheetData>
   <dataValidations count="16">
-    <dataValidation sqref="B33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B33" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: +X, -X, +Y, -Y" type="list" errorStyle="stop">
       <formula1>"+X,-X,+Y,-Y"</formula1>
     </dataValidation>
-    <dataValidation sqref="A46:A85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A46:A85" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: 1, 0" type="list" errorStyle="stop">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="C46:C85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C46:C85" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: boom, rear_leg, front_leg, platform" type="list" errorStyle="stop">
       <formula1>"boom,rear_leg,front_leg,platform"</formula1>
     </dataValidation>
-    <dataValidation sqref="D46:D85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D46:D85" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: boom_local, global" type="list" errorStyle="stop">
       <formula1>"boom_local,global"</formula1>
     </dataValidation>
-    <dataValidation sqref="A92:A131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A92:A131" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: 1, 0" type="list" errorStyle="stop">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="C92:C131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C92:C131" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: boom, rear_leg, front_leg, platform" type="list" errorStyle="stop">
       <formula1>"boom,rear_leg,front_leg,platform"</formula1>
     </dataValidation>
-    <dataValidation sqref="D92:D131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D92:D131" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: boom_local, global" type="list" errorStyle="stop">
       <formula1>"boom_local,global"</formula1>
     </dataValidation>
-    <dataValidation sqref="A138:A217" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A138:A217" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: 1, 0" type="list" errorStyle="stop">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="C138:C217" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C138:C217" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: boom, rear_leg, front_leg, platform" type="list" errorStyle="stop">
       <formula1>"boom,rear_leg,front_leg,platform"</formula1>
     </dataValidation>
-    <dataValidation sqref="D138:D217" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D138:D217" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: boom_local, global, hanging" type="list" errorStyle="stop">
       <formula1>"boom_local,global,hanging"</formula1>
     </dataValidation>
-    <dataValidation sqref="K138:K217" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K138:K217" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: 1, 0" type="list" errorStyle="stop">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="A224:A283" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A224:A283" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: 1, 0" type="list" errorStyle="stop">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="A290:A297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A290:A297" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: 1, 0" type="list" errorStyle="stop">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="C290:C297" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C290:C297" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: fixed, solve" type="list" errorStyle="stop">
       <formula1>"fixed,solve"</formula1>
     </dataValidation>
-    <dataValidation sqref="A304:A311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A304:A311" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: 1, 0" type="list" errorStyle="stop">
       <formula1>"1,0"</formula1>
     </dataValidation>
-    <dataValidation sqref="O304:O311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O304:O311" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: 1, 0" type="list" errorStyle="stop">
       <formula1>"1,0"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7289,7 +7289,7 @@
         </is>
       </c>
       <c r="B20" s="3">
-        <f>IFERROR(INDEX(Inputs!$D$304:$D$311,MATCH(Inputs!$B$26,Inputs!$B$304:$B$311,0))&amp;"","")</f>
+        <f>IFERROR(INDEX(Inputs!$D$304:$D$311,MATCH(Inputs!$B$26&amp;"",Loads!$B$139:$B$146,0))&amp;"","")</f>
         <v/>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -7342,7 +7342,7 @@
         </is>
       </c>
       <c r="B23" s="3">
-        <f>IF(Geometry!$B$22&lt;&gt;"",Geometry!$B$22,IFERROR(INDEX(Inputs!$E$304:$E$311,MATCH(Inputs!$B$26,Inputs!$B$304:$B$311,0))&amp;"",""))</f>
+        <f>IF(Geometry!$B$22&lt;&gt;"",Geometry!$B$22,IFERROR(INDEX(Inputs!$E$304:$E$311,MATCH(Inputs!$B$26&amp;"",Loads!$B$139:$B$146,0))&amp;"",""))</f>
         <v/>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -12493,7 +12493,7 @@
         </is>
       </c>
       <c r="B28" s="3">
-        <f>IFERROR(INDEX(Loads!$C$139:$C$146,MATCH(Inputs!$B$26,Loads!$B$139:$B$146,0))&amp;"","")</f>
+        <f>IFERROR(INDEX(Loads!$C$139:$C$146,MATCH(Inputs!$B$26&amp;"",Loads!$B$139:$B$146,0))&amp;"","")</f>
         <v/>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -17058,7 +17058,7 @@
         <v/>
       </c>
       <c r="D139" s="3">
-        <f>IF(AND(Loads!$A$139=1,Loads!$B$139&lt;&gt;"",Loads!$B$139=Inputs!$B$26),1,0)</f>
+        <f>IF(AND(Loads!$A$139=1,Loads!$B$139&lt;&gt;"",Loads!$B$139=Inputs!$B$26&amp;""),1,0)</f>
         <v/>
       </c>
       <c r="E139" s="3">
@@ -17108,7 +17108,7 @@
         <v/>
       </c>
       <c r="D140" s="3">
-        <f>IF(AND(Loads!$A$140=1,Loads!$B$140&lt;&gt;"",Loads!$B$140=Inputs!$B$26),1,0)</f>
+        <f>IF(AND(Loads!$A$140=1,Loads!$B$140&lt;&gt;"",Loads!$B$140=Inputs!$B$26&amp;""),1,0)</f>
         <v/>
       </c>
       <c r="E140" s="3">
@@ -17158,7 +17158,7 @@
         <v/>
       </c>
       <c r="D141" s="3">
-        <f>IF(AND(Loads!$A$141=1,Loads!$B$141&lt;&gt;"",Loads!$B$141=Inputs!$B$26),1,0)</f>
+        <f>IF(AND(Loads!$A$141=1,Loads!$B$141&lt;&gt;"",Loads!$B$141=Inputs!$B$26&amp;""),1,0)</f>
         <v/>
       </c>
       <c r="E141" s="3">
@@ -17208,7 +17208,7 @@
         <v/>
       </c>
       <c r="D142" s="3">
-        <f>IF(AND(Loads!$A$142=1,Loads!$B$142&lt;&gt;"",Loads!$B$142=Inputs!$B$26),1,0)</f>
+        <f>IF(AND(Loads!$A$142=1,Loads!$B$142&lt;&gt;"",Loads!$B$142=Inputs!$B$26&amp;""),1,0)</f>
         <v/>
       </c>
       <c r="E142" s="3">
@@ -17258,7 +17258,7 @@
         <v/>
       </c>
       <c r="D143" s="3">
-        <f>IF(AND(Loads!$A$143=1,Loads!$B$143&lt;&gt;"",Loads!$B$143=Inputs!$B$26),1,0)</f>
+        <f>IF(AND(Loads!$A$143=1,Loads!$B$143&lt;&gt;"",Loads!$B$143=Inputs!$B$26&amp;""),1,0)</f>
         <v/>
       </c>
       <c r="E143" s="3">
@@ -17308,7 +17308,7 @@
         <v/>
       </c>
       <c r="D144" s="3">
-        <f>IF(AND(Loads!$A$144=1,Loads!$B$144&lt;&gt;"",Loads!$B$144=Inputs!$B$26),1,0)</f>
+        <f>IF(AND(Loads!$A$144=1,Loads!$B$144&lt;&gt;"",Loads!$B$144=Inputs!$B$26&amp;""),1,0)</f>
         <v/>
       </c>
       <c r="E144" s="3">
@@ -17358,7 +17358,7 @@
         <v/>
       </c>
       <c r="D145" s="3">
-        <f>IF(AND(Loads!$A$145=1,Loads!$B$145&lt;&gt;"",Loads!$B$145=Inputs!$B$26),1,0)</f>
+        <f>IF(AND(Loads!$A$145=1,Loads!$B$145&lt;&gt;"",Loads!$B$145=Inputs!$B$26&amp;""),1,0)</f>
         <v/>
       </c>
       <c r="E145" s="3">
@@ -17408,7 +17408,7 @@
         <v/>
       </c>
       <c r="D146" s="3">
-        <f>IF(AND(Loads!$A$146=1,Loads!$B$146&lt;&gt;"",Loads!$B$146=Inputs!$B$26),1,0)</f>
+        <f>IF(AND(Loads!$A$146=1,Loads!$B$146&lt;&gt;"",Loads!$B$146=Inputs!$B$26&amp;""),1,0)</f>
         <v/>
       </c>
       <c r="E146" s="3">
@@ -36865,7 +36865,7 @@
         </is>
       </c>
       <c r="B26" s="3">
-        <f>IF(Inputs!$B$26="",0,IFERROR(MATCH(Inputs!$B$26,Loads!$B$139:$B$146,0),0))</f>
+        <f>IF(Inputs!$B$26="",0,IFERROR(MATCH(Inputs!$B$26&amp;"",Loads!$B$139:$B$146,0),0))</f>
         <v/>
       </c>
       <c r="C26" t="inlineStr">
@@ -45570,7 +45570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -45593,7 +45593,7 @@
         </is>
       </c>
       <c r="C3" s="3">
-        <f>SUM(C6:C20)</f>
+        <f>SUM(C6:C22)</f>
         <v/>
       </c>
       <c r="D3" s="3">
@@ -45635,7 +45635,7 @@
         </is>
       </c>
       <c r="C6" s="3">
-        <f>SUM($D$25:$D$30)</f>
+        <f>SUM($D$27:$D$32)</f>
         <v/>
       </c>
       <c r="D6" s="3">
@@ -45646,16 +45646,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>duplicate_ids</t>
+          <t>mirror</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Active rows whose id is used by another active row of the same table</t>
+          <t>Inputs tables with rows inserted or deleted (never do that: use spare rows), or a calculation sheet whose rows no longer follow the Inputs rows</t>
         </is>
       </c>
       <c r="C7" s="3">
-        <f>SUMPRODUCT((Inputs!$A$46:$A$85=1)*(Inputs!$B$46:$B$85&lt;&gt;"")*(COUNTIFS(Inputs!$B$46:$B$85,Inputs!$B$46:$B$85,Inputs!$A$46:$A$85,1)&gt;1))+SUMPRODUCT((Inputs!$A$92:$A$131=1)*(Inputs!$B$92:$B$131&lt;&gt;"")*(COUNTIFS(Inputs!$B$92:$B$131,Inputs!$B$92:$B$131,Inputs!$A$92:$A$131,1)&gt;1))+SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$B$138:$B$217&lt;&gt;"")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$B$138:$B$217,Inputs!$A$138:$A$217,1)&gt;1))+SUMPRODUCT((Inputs!$A$290:$A$297=1)*(Inputs!$B$290:$B$297&lt;&gt;"")*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$B$290:$B$297,Inputs!$A$290:$A$297,1)&gt;1))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(Inputs!$B$304:$B$311&lt;&gt;"")*(COUNTIFS(Inputs!$B$304:$B$311,Inputs!$B$304:$B$311,Inputs!$A$304:$A$311,1)&gt;1))</f>
+        <f>IFERROR(1*(ROWS(Inputs!$A$46:$A$85)&lt;&gt;40)+1*(SUM(Inputs!$A$46:$A$85)&lt;&gt;SUM(Loads!$A$33:$A$72)),1)+IFERROR(1*(ROWS(Inputs!$A$46:$A$85)&lt;&gt;40)+1*(SUM(Inputs!$A$46:$A$85)&lt;&gt;SUM(OutOfPlane!$A$39:$A$78)),1)+IFERROR(1*(ROWS(Inputs!$A$92:$A$131)&lt;&gt;40)+1*(SUM(Inputs!$A$92:$A$131)&lt;&gt;SUM(Loads!$A$79:$A$118)),1)+IFERROR(1*(ROWS(Inputs!$A$92:$A$131)&lt;&gt;40)+1*(SUM(Inputs!$A$92:$A$131)&lt;&gt;SUM(OutOfPlane!$A$171:$A$210)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(Geometry!$A$58:$A$137)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(Loads!$A$219:$A$298)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(OutOfPlane!$A$85:$A$164)),1)+IFERROR(1*(ROWS(Inputs!$A$224:$A$283)&lt;&gt;60)+1*(SUM(Inputs!$A$224:$A$283)&lt;&gt;SUM(Loads!$A$153:$A$212)),1)+IFERROR(1*(ROWS(Inputs!$A$290:$A$297)&lt;&gt;8)+1*(SUM(Inputs!$A$290:$A$297)&lt;&gt;SUM(Loads!$A$125:$A$132)),1)+IFERROR(1*(ROWS(Inputs!$A$304:$A$311)&lt;&gt;8)+1*(SUM(Inputs!$A$304:$A$311)&lt;&gt;SUM(Loads!$A$139:$A$146)),1)+IFERROR(1*(ROWS(Inputs!$A$304:$A$311)&lt;&gt;8)+1*(SUM(Inputs!$A$304:$A$311)&lt;&gt;SUM(Results!$A$19:$A$26)),1)</f>
         <v/>
       </c>
       <c r="D7" s="3">
@@ -45666,16 +45666,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>blank_ids</t>
+          <t>duplicate_ids</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Active rows with a blank id (or blank rope id on a segment)</t>
+          <t>Active node, rope or hoist rows whose id is used by another active row of the same table (mass-point and wind-area ids are labels only)</t>
         </is>
       </c>
       <c r="C8" s="3">
-        <f>SUMPRODUCT((Inputs!$A$46:$A$85=1)*(Inputs!$B$46:$B$85=""))+SUMPRODUCT((Inputs!$A$92:$A$131=1)*(Inputs!$B$92:$B$131=""))+SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$B$138:$B$217=""))+SUMPRODUCT((Inputs!$A$290:$A$297=1)*(Inputs!$B$290:$B$297=""))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(Inputs!$B$304:$B$311=""))+SUMPRODUCT((Inputs!$A$224:$A$283=1)*(Inputs!$B$224:$B$283=""))</f>
+        <f>SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$B$138:$B$217&lt;&gt;"")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$B$138:$B$217,Inputs!$A$138:$A$217,1)&gt;1))+SUMPRODUCT((Inputs!$A$290:$A$297=1)*(Inputs!$B$290:$B$297&lt;&gt;"")*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$B$290:$B$297,Inputs!$A$290:$A$297,1)&gt;1))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(Inputs!$B$304:$B$311&lt;&gt;"")*(COUNTIFS(Inputs!$B$304:$B$311,Inputs!$B$304:$B$311,Inputs!$A$304:$A$311,1)&gt;1))</f>
         <v/>
       </c>
       <c r="D8" s="3">
@@ -45686,16 +45686,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>node_references</t>
+          <t>blank_ids</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>References to a missing or inactive node (segment ends, hoist hook/support nodes, hanging nodes' parent)</t>
+          <t>Active rows with a blank id (or blank rope id on a segment)</t>
         </is>
       </c>
       <c r="C9" s="3">
-        <f>SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$C$224:$C$283,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$D$224:$D$283,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$D$304:$D$311,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(Inputs!$E$304:$E$311&lt;&gt;"")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$E$304:$E$311,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="hanging")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$I$138:$I$217,Inputs!$A$138:$A$217,1)=0))</f>
+        <f>SUMPRODUCT((Inputs!$A$46:$A$85=1)*(Inputs!$B$46:$B$85=""))+SUMPRODUCT((Inputs!$A$92:$A$131=1)*(Inputs!$B$92:$B$131=""))+SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$B$138:$B$217=""))+SUMPRODUCT((Inputs!$A$290:$A$297=1)*(Inputs!$B$290:$B$297=""))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(Inputs!$B$304:$B$311=""))+SUMPRODUCT((Inputs!$A$224:$A$283=1)*(Inputs!$B$224:$B$283=""))</f>
         <v/>
       </c>
       <c r="D9" s="3">
@@ -45706,16 +45706,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>rope_references</t>
+          <t>invalid_values</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Segments or hoists referencing a missing or inactive rope</t>
+          <t>Cells outside their allowed values: Active not blank/0/1; on active rows a 1/0 column not 0/1, or a body, frame or role not one of its list choices (a typo drops the row)</t>
         </is>
       </c>
       <c r="C10" s="3">
-        <f>SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$B$224:$B$283,Inputs!$A$290:$A$297,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$C$304:$C$311,Inputs!$A$290:$A$297,1)=0))</f>
+        <f>SUMPRODUCT(1*(Inputs!$A$46:$A$85&lt;&gt;"")*(Inputs!$A$46:$A$85&lt;&gt;0)*(Inputs!$A$46:$A$85&lt;&gt;1))+SUMPRODUCT(1*(Inputs!$A$46:$A$85=1)*(Inputs!$C$46:$C$85&lt;&gt;"boom")*(Inputs!$C$46:$C$85&lt;&gt;"rear_leg")*(Inputs!$C$46:$C$85&lt;&gt;"front_leg")*(Inputs!$C$46:$C$85&lt;&gt;"platform"))+SUMPRODUCT(1*(Inputs!$A$46:$A$85=1)*(Inputs!$D$46:$D$85&lt;&gt;"boom_local")*(Inputs!$D$46:$D$85&lt;&gt;"global"))+SUMPRODUCT(1*(Inputs!$A$92:$A$131&lt;&gt;"")*(Inputs!$A$92:$A$131&lt;&gt;0)*(Inputs!$A$92:$A$131&lt;&gt;1))+SUMPRODUCT(1*(Inputs!$A$92:$A$131=1)*(Inputs!$C$92:$C$131&lt;&gt;"boom")*(Inputs!$C$92:$C$131&lt;&gt;"rear_leg")*(Inputs!$C$92:$C$131&lt;&gt;"front_leg")*(Inputs!$C$92:$C$131&lt;&gt;"platform"))+SUMPRODUCT(1*(Inputs!$A$92:$A$131=1)*(Inputs!$D$92:$D$131&lt;&gt;"boom_local")*(Inputs!$D$92:$D$131&lt;&gt;"global"))+SUMPRODUCT(1*(Inputs!$A$138:$A$217&lt;&gt;"")*(Inputs!$A$138:$A$217&lt;&gt;0)*(Inputs!$A$138:$A$217&lt;&gt;1))+SUMPRODUCT(1*(Inputs!$A$138:$A$217=1)*(Inputs!$C$138:$C$217&lt;&gt;"boom")*(Inputs!$C$138:$C$217&lt;&gt;"rear_leg")*(Inputs!$C$138:$C$217&lt;&gt;"front_leg")*(Inputs!$C$138:$C$217&lt;&gt;"platform"))+SUMPRODUCT(1*(Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217&lt;&gt;"boom_local")*(Inputs!$D$138:$D$217&lt;&gt;"global")*(Inputs!$D$138:$D$217&lt;&gt;"hanging"))+SUMPRODUCT(1*(Inputs!$A$138:$A$217=1)*(Inputs!$K$138:$K$217&lt;&gt;"")*(Inputs!$K$138:$K$217&lt;&gt;0)*(Inputs!$K$138:$K$217&lt;&gt;1))+SUMPRODUCT(1*(Inputs!$A$224:$A$283&lt;&gt;"")*(Inputs!$A$224:$A$283&lt;&gt;0)*(Inputs!$A$224:$A$283&lt;&gt;1))+SUMPRODUCT(1*(Inputs!$A$290:$A$297&lt;&gt;"")*(Inputs!$A$290:$A$297&lt;&gt;0)*(Inputs!$A$290:$A$297&lt;&gt;1))+SUMPRODUCT(1*(Inputs!$A$290:$A$297=1)*(Inputs!$C$290:$C$297&lt;&gt;"fixed")*(Inputs!$C$290:$C$297&lt;&gt;"solve"))+SUMPRODUCT(1*(Inputs!$A$304:$A$311&lt;&gt;"")*(Inputs!$A$304:$A$311&lt;&gt;0)*(Inputs!$A$304:$A$311&lt;&gt;1))+SUMPRODUCT(1*(Inputs!$A$304:$A$311=1)*(Inputs!$O$304:$O$311&lt;&gt;"")*(Inputs!$O$304:$O$311&lt;&gt;0)*(Inputs!$O$304:$O$311&lt;&gt;1))</f>
         <v/>
       </c>
       <c r="D10" s="3">
@@ -45726,16 +45726,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>hoist_without_segments</t>
+          <t>node_references</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Active hoists whose rope has no active segment</t>
+          <t>References to a missing or inactive node (segment ends, hoist hook/support nodes, hanging nodes' parent)</t>
         </is>
       </c>
       <c r="C11" s="3">
-        <f>SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$224:$B$283,Inputs!$C$304:$C$311,Inputs!$A$224:$A$283,1)=0))</f>
+        <f>SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$C$224:$C$283,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$D$224:$D$283,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$D$304:$D$311,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(Inputs!$E$304:$E$311&lt;&gt;"")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$E$304:$E$311,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="hanging")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$I$138:$I$217,Inputs!$A$138:$A$217,1)=0))</f>
         <v/>
       </c>
       <c r="D11" s="3">
@@ -45746,16 +45746,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>multiple_solve_ropes</t>
+          <t>rope_references</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Active solve ropes beyond the first (exactly one is allowed)</t>
+          <t>Segments or hoists referencing a missing or inactive rope</t>
         </is>
       </c>
       <c r="C12" s="3">
-        <f>MAX(0,COUNTIFS(Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"solve")-1)</f>
+        <f>SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$B$224:$B$283,Inputs!$A$290:$A$297,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$C$304:$C$311,Inputs!$A$290:$A$297,1)=0))</f>
         <v/>
       </c>
       <c r="D12" s="3">
@@ -45766,16 +45766,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>no_solve_rope</t>
+          <t>hoist_without_segments</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1 if no active rope has role solve (the app shows no results then)</t>
+          <t>Active hoists whose rope has no active segment</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>IF(COUNTIFS(Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"solve")=0,1,0)</f>
+        <f>SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$224:$B$283,Inputs!$C$304:$C$311,Inputs!$A$224:$A$283,1)=0))</f>
         <v/>
       </c>
       <c r="D13" s="3">
@@ -45786,16 +45786,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>scene_hoist</t>
+          <t>multiple_solve_ropes</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1 if the scene hoist is not an active hoist with a fixed rope</t>
+          <t>Active solve ropes beyond the first (exactly one is allowed)</t>
         </is>
       </c>
       <c r="C14" s="3">
-        <f>IF(COUNTIFS(Inputs!$B$304:$B$311,Inputs!$B$26,Inputs!$A$304:$A$311,1)=0,1,IF(COUNTIFS(Inputs!$B$290:$B$297,INDEX(Inputs!$C$304:$C$311,MATCH(Inputs!$B$26,Inputs!$B$304:$B$311,0)),Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"fixed")=0,1,0))</f>
+        <f>MAX(0,COUNTIFS(Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"solve")-1)</f>
         <v/>
       </c>
       <c r="D14" s="3">
@@ -45806,16 +45806,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>wind_direction</t>
+          <t>no_solve_rope</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1 if the scene wind direction is not +X, -X, +Y or -Y</t>
+          <t>1 if no active rope has role solve (the app shows no results then)</t>
         </is>
       </c>
       <c r="C15" s="3">
-        <f>IF(OR(Inputs!$B$33="+X",Inputs!$B$33="-X",Inputs!$B$33="+Y",Inputs!$B$33="-Y"),0,1)</f>
+        <f>IF(COUNTIFS(Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"solve")=0,1,0)</f>
         <v/>
       </c>
       <c r="D15" s="3">
@@ -45826,16 +45826,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fixed_nodes_missing</t>
+          <t>scene_hoist</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Fixed structure node ids with no active node row</t>
+          <t>1 if the scene hoist is not an active hoist with a fixed rope</t>
         </is>
       </c>
       <c r="C16" s="3">
-        <f>COUNTIF($B$34:$B$42,0)</f>
+        <f>IF(COUNTIFS(Inputs!$B$304:$B$311,Inputs!$B$26,Inputs!$A$304:$A$311,1)=0,1,IF(COUNTIFS(Inputs!$B$290:$B$297,IFERROR(INDEX(Inputs!$C$304:$C$311,MATCH(Inputs!$B$26&amp;"",Loads!$B$139:$B$146,0)),""),Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"fixed")=0,1,0))</f>
         <v/>
       </c>
       <c r="D16" s="3">
@@ -45846,16 +45846,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>hanging_chain</t>
+          <t>wind_direction</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hanging nodes whose parent is itself hanging (only one level is resolved)</t>
+          <t>1 if the scene wind direction is not +X, -X, +Y or -Y</t>
         </is>
       </c>
       <c r="C17" s="3">
-        <f>SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="hanging")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$I$138:$I$217,Inputs!$D$138:$D$217,"hanging",Inputs!$A$138:$A$217,1)&gt;0))</f>
+        <f>IF(OR(Inputs!$B$33="+X",Inputs!$B$33="-X",Inputs!$B$33="+Y",Inputs!$B$33="-Y"),0,1)</f>
         <v/>
       </c>
       <c r="D17" s="3">
@@ -45866,16 +45866,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>singular_matrix</t>
+          <t>fixed_nodes_missing</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Singular Statics systems (boom 3x3, leg frame 6x6); the boom one is singular without a solve rope</t>
+          <t>Fixed structure node ids with no active node row</t>
         </is>
       </c>
       <c r="C18" s="3">
-        <f>Statics!$B$41+Statics!$B$62</f>
+        <f>COUNTIF($B$36:$B$44,0)</f>
         <v/>
       </c>
       <c r="D18" s="3">
@@ -45886,16 +45886,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>zero_boom_width</t>
+          <t>hanging_chain</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>1 if the boom width is not &gt; 0 (the app rejects it; the out-of-plane split divides by it, so Results shows a message)</t>
+          <t>Hanging nodes whose parent is itself hanging (only one level is resolved)</t>
         </is>
       </c>
       <c r="C19" s="3">
-        <f>IF(OutOfPlane!$B$21=1,0,1)</f>
+        <f>SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="hanging")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$I$138:$I$217,Inputs!$D$138:$D$217,"hanging",Inputs!$A$138:$A$217,1)&gt;0))</f>
         <v/>
       </c>
       <c r="D19" s="3">
@@ -45906,16 +45906,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>invalid_bearing_diameter</t>
+          <t>singular_matrix</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>1 if the slewing bearing diameter is typed but not a number &gt; 0 (blank is allowed and hides the bearing line-load rows)</t>
+          <t>Singular Statics systems (boom 3x3, leg frame 6x6); the boom one is singular without a solve rope</t>
         </is>
       </c>
       <c r="C20" s="3">
-        <f>IF(Inputs!$B$13="",0,IF(ISNUMBER(Inputs!$B$13),IF(Inputs!$B$13&gt;0,0,1),1))</f>
+        <f>Statics!$B$41+Statics!$B$62</f>
         <v/>
       </c>
       <c r="D20" s="3">
@@ -45923,85 +45923,87 @@
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>zero_boom_width</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1 if the boom width is not &gt; 0 (the app rejects it; the out-of-plane split divides by it, so Results shows a message)</t>
+        </is>
+      </c>
+      <c r="C21" s="3">
+        <f>IF(OutOfPlane!$B$21=1,0,1)</f>
+        <v/>
+      </c>
+      <c r="D21" s="3">
+        <f>IF(C21=0,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>invalid_bearing_diameter</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1 if the slewing bearing diameter is typed but not a number &gt; 0 (blank is allowed and hides the bearing line-load rows)</t>
+        </is>
+      </c>
+      <c r="C22" s="3">
+        <f>IF(Inputs!$B$13="",0,IF(ISNUMBER(Inputs!$B$13),IF(Inputs!$B$13&gt;0,0,1),1))</f>
+        <v/>
+      </c>
+      <c r="D22" s="3">
+        <f>IF(C22=0,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Overflow per table</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Not written</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>Typed in guard row</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>mass_points</t>
-        </is>
-      </c>
-      <c r="B25" s="3">
-        <f>Inputs!$G$43</f>
-        <v/>
-      </c>
-      <c r="C25" s="3">
-        <f>COUNTA(Inputs!$A$86:$K$86)</f>
-        <v/>
-      </c>
-      <c r="D25" s="3">
-        <f>B25+C25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>wind_areas</t>
-        </is>
-      </c>
-      <c r="B26" s="3">
-        <f>Inputs!$G$89</f>
-        <v/>
-      </c>
-      <c r="C26" s="3">
-        <f>COUNTA(Inputs!$A$132:$K$132)</f>
-        <v/>
-      </c>
-      <c r="D26" s="3">
-        <f>B26+C26</f>
-        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>nodes</t>
+          <t>mass_points</t>
         </is>
       </c>
       <c r="B27" s="3">
-        <f>Inputs!$G$135</f>
+        <f>Inputs!$G$43</f>
         <v/>
       </c>
       <c r="C27" s="3">
-        <f>COUNTA(Inputs!$A$218:$K$218)</f>
+        <f>COUNTA(Inputs!$A$86:$K$86)</f>
         <v/>
       </c>
       <c r="D27" s="3">
@@ -46012,15 +46014,15 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>segments</t>
+          <t>wind_areas</t>
         </is>
       </c>
       <c r="B28" s="3">
-        <f>Inputs!$G$221</f>
+        <f>Inputs!$G$89</f>
         <v/>
       </c>
       <c r="C28" s="3">
-        <f>COUNTA(Inputs!$A$284:$E$284)</f>
+        <f>COUNTA(Inputs!$A$132:$K$132)</f>
         <v/>
       </c>
       <c r="D28" s="3">
@@ -46031,15 +46033,15 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ropes</t>
+          <t>nodes</t>
         </is>
       </c>
       <c r="B29" s="3">
-        <f>Inputs!$G$287</f>
+        <f>Inputs!$G$135</f>
         <v/>
       </c>
       <c r="C29" s="3">
-        <f>COUNTA(Inputs!$A$298:$C$298)</f>
+        <f>COUNTA(Inputs!$A$218:$K$218)</f>
         <v/>
       </c>
       <c r="D29" s="3">
@@ -46050,15 +46052,15 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>hoists</t>
+          <t>segments</t>
         </is>
       </c>
       <c r="B30" s="3">
-        <f>Inputs!$G$301</f>
+        <f>Inputs!$G$221</f>
         <v/>
       </c>
       <c r="C30" s="3">
-        <f>COUNTA(Inputs!$A$312:$Q$312)</f>
+        <f>COUNTA(Inputs!$A$284:$E$284)</f>
         <v/>
       </c>
       <c r="D30" s="3">
@@ -46066,39 +46068,55 @@
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ropes</t>
+        </is>
+      </c>
+      <c r="B31" s="3">
+        <f>Inputs!$G$287</f>
+        <v/>
+      </c>
+      <c r="C31" s="3">
+        <f>COUNTA(Inputs!$A$298:$C$298)</f>
+        <v/>
+      </c>
+      <c r="D31" s="3">
+        <f>B31+C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>hoists</t>
+        </is>
+      </c>
+      <c r="B32" s="3">
+        <f>Inputs!$G$301</f>
+        <v/>
+      </c>
+      <c r="C32" s="3">
+        <f>COUNTA(Inputs!$A$312:$Q$312)</f>
+        <v/>
+      </c>
+      <c r="D32" s="3">
+        <f>B32+C32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Fixed structure nodes (active rows with this id)</t>
         </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>boom_heel</t>
-        </is>
-      </c>
-      <c r="B34" s="3">
-        <f>COUNTIFS(Inputs!$B$138:$B$217,A34,Inputs!$A$138:$A$217,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>platform_heel</t>
-        </is>
-      </c>
-      <c r="B35" s="3">
-        <f>COUNTIFS(Inputs!$B$138:$B$217,A35,Inputs!$A$138:$A$217,1)</f>
-        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>rear_top</t>
+          <t>boom_heel</t>
         </is>
       </c>
       <c r="B36" s="3">
@@ -46109,7 +46127,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>front_top</t>
+          <t>platform_heel</t>
         </is>
       </c>
       <c r="B37" s="3">
@@ -46120,7 +46138,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>rear_base</t>
+          <t>rear_top</t>
         </is>
       </c>
       <c r="B38" s="3">
@@ -46131,7 +46149,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>platform_rear</t>
+          <t>front_top</t>
         </is>
       </c>
       <c r="B39" s="3">
@@ -46142,7 +46160,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>front_base</t>
+          <t>rear_base</t>
         </is>
       </c>
       <c r="B40" s="3">
@@ -46153,7 +46171,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>platform_front</t>
+          <t>platform_rear</t>
         </is>
       </c>
       <c r="B41" s="3">
@@ -46164,7 +46182,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>platform_base</t>
+          <t>front_base</t>
         </is>
       </c>
       <c r="B42" s="3">
@@ -46172,8 +46190,30 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>platform_front</t>
+        </is>
+      </c>
+      <c r="B43" s="3">
+        <f>COUNTIFS(Inputs!$B$138:$B$217,A43,Inputs!$A$138:$A$217,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>platform_base</t>
+        </is>
+      </c>
+      <c r="B44" s="3">
+        <f>COUNTIFS(Inputs!$B$138:$B$217,A44,Inputs!$A$138:$A$217,1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C6:C20">
+  <conditionalFormatting sqref="C6:C22">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Workbook checks: boom_local on a non-boom body, rows inserted at a table's start or end (mirror), bearing diameter validation; regenerate 22689 workbook
</commit_message>
<xml_diff>
--- a/docs/crane-statics-validation-22689.xlsx
+++ b/docs/crane-statics-validation-22689.xlsx
@@ -6989,7 +6989,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="16">
+  <dataValidations count="17">
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Type a number &gt; 0, or leave the cell blank." type="decimal" errorStyle="stop" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
     <dataValidation sqref="B33" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Pick one of: +X, -X, +Y, -Y" type="list" errorStyle="stop">
       <formula1>"+X,-X,+Y,-Y"</formula1>
     </dataValidation>
@@ -45372,7 +45375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -45395,7 +45398,7 @@
         </is>
       </c>
       <c r="C3" s="3">
-        <f>SUM(C6:C22)</f>
+        <f>SUM(C6:C23)</f>
         <v/>
       </c>
       <c r="D3" s="3">
@@ -45437,7 +45440,7 @@
         </is>
       </c>
       <c r="C6" s="3">
-        <f>SUM($D$27:$D$32)</f>
+        <f>SUM($D$28:$D$33)</f>
         <v/>
       </c>
       <c r="D6" s="3">
@@ -45453,11 +45456,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Inputs tables with rows inserted or deleted (never do that: use spare rows), or a calculation sheet whose rows no longer follow the Inputs rows</t>
+          <t>Inputs tables with rows inserted or deleted (never do that: use spare rows), including a row inserted above the first data row or above the guard row, or a calculation sheet whose rows no longer follow the Inputs rows</t>
         </is>
       </c>
       <c r="C7" s="3">
-        <f>IFERROR(1*(ROWS(Inputs!$A$46:$A$85)&lt;&gt;40)+1*(SUM(Inputs!$A$46:$A$85)&lt;&gt;SUM(Loads!$A$33:$A$72)),1)+IFERROR(1*(ROWS(Inputs!$A$46:$A$85)&lt;&gt;40)+1*(SUM(Inputs!$A$46:$A$85)&lt;&gt;SUM(OutOfPlane!$A$38:$A$77)),1)+IFERROR(1*(ROWS(Inputs!$A$92:$A$131)&lt;&gt;40)+1*(SUM(Inputs!$A$92:$A$131)&lt;&gt;SUM(Loads!$A$79:$A$118)),1)+IFERROR(1*(ROWS(Inputs!$A$92:$A$131)&lt;&gt;40)+1*(SUM(Inputs!$A$92:$A$131)&lt;&gt;SUM(OutOfPlane!$A$170:$A$209)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(Geometry!$A$58:$A$137)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(Loads!$A$219:$A$298)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(OutOfPlane!$A$84:$A$163)),1)+IFERROR(1*(ROWS(Inputs!$A$224:$A$283)&lt;&gt;60)+1*(SUM(Inputs!$A$224:$A$283)&lt;&gt;SUM(Loads!$A$153:$A$212)),1)+IFERROR(1*(ROWS(Inputs!$A$290:$A$297)&lt;&gt;8)+1*(SUM(Inputs!$A$290:$A$297)&lt;&gt;SUM(Loads!$A$125:$A$132)),1)+IFERROR(1*(ROWS(Inputs!$A$304:$A$311)&lt;&gt;8)+1*(SUM(Inputs!$A$304:$A$311)&lt;&gt;SUM(Loads!$A$139:$A$146)),1)+IFERROR(1*(ROWS(Inputs!$A$304:$A$311)&lt;&gt;8)+1*(SUM(Inputs!$A$304:$A$311)&lt;&gt;SUM(Results!$A$19:$A$26)),1)</f>
+        <f>IFERROR(1*(ROWS(Inputs!$A$46:$A$85)&lt;&gt;40)+1*(SUM(Inputs!$A$46:$A$85)&lt;&gt;SUM(Loads!$A$33:$A$72)),1)+IFERROR(1*(ROWS(Inputs!$A$46:$A$85)&lt;&gt;40)+1*(SUM(Inputs!$A$46:$A$85)&lt;&gt;SUM(OutOfPlane!$A$38:$A$77)),1)+IFERROR(1*(ROWS(Inputs!$A$92:$A$131)&lt;&gt;40)+1*(SUM(Inputs!$A$92:$A$131)&lt;&gt;SUM(Loads!$A$79:$A$118)),1)+IFERROR(1*(ROWS(Inputs!$A$92:$A$131)&lt;&gt;40)+1*(SUM(Inputs!$A$92:$A$131)&lt;&gt;SUM(OutOfPlane!$A$170:$A$209)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(Geometry!$A$58:$A$137)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(Loads!$A$219:$A$298)),1)+IFERROR(1*(ROWS(Inputs!$A$138:$A$217)&lt;&gt;80)+1*(SUM(Inputs!$A$138:$A$217)&lt;&gt;SUM(OutOfPlane!$A$84:$A$163)),1)+IFERROR(1*(ROWS(Inputs!$A$224:$A$283)&lt;&gt;60)+1*(SUM(Inputs!$A$224:$A$283)&lt;&gt;SUM(Loads!$A$153:$A$212)),1)+IFERROR(1*(ROWS(Inputs!$A$290:$A$297)&lt;&gt;8)+1*(SUM(Inputs!$A$290:$A$297)&lt;&gt;SUM(Loads!$A$125:$A$132)),1)+IFERROR(1*(ROWS(Inputs!$A$304:$A$311)&lt;&gt;8)+1*(SUM(Inputs!$A$304:$A$311)&lt;&gt;SUM(Loads!$A$139:$A$146)),1)+IFERROR(1*(ROWS(Inputs!$A$304:$A$311)&lt;&gt;8)+1*(SUM(Inputs!$A$304:$A$311)&lt;&gt;SUM(Results!$A$19:$A$26)),1)+IFERROR(1*(ROW(Inputs!$A$86)-ROW(Inputs!$A$45)&lt;&gt;41),1)+IFERROR(1*(ROW(Inputs!$A$132)-ROW(Inputs!$A$91)&lt;&gt;41),1)+IFERROR(1*(ROW(Inputs!$A$218)-ROW(Inputs!$A$137)&lt;&gt;81),1)+IFERROR(1*(ROW(Inputs!$A$284)-ROW(Inputs!$A$223)&lt;&gt;61),1)+IFERROR(1*(ROW(Inputs!$A$298)-ROW(Inputs!$A$289)&lt;&gt;9),1)+IFERROR(1*(ROW(Inputs!$A$312)-ROW(Inputs!$A$303)&lt;&gt;9),1)</f>
         <v/>
       </c>
       <c r="D7" s="3">
@@ -45528,16 +45531,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>node_references</t>
+          <t>boom_local_non_boom</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>References to a missing or inactive node (segment ends, hoist hook/support nodes, hanging nodes' parent)</t>
+          <t>Active mass-point, wind-area or node rows with frame boom_local on a body other than boom (the app ignores u/v/w there and uses x/z)</t>
         </is>
       </c>
       <c r="C11" s="3">
-        <f>SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$C$224:$C$283,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$D$224:$D$283,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$D$304:$D$311,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(Inputs!$E$304:$E$311&lt;&gt;"")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$E$304:$E$311,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="hanging")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$I$138:$I$217,Inputs!$A$138:$A$217,1)=0))</f>
+        <f>SUMPRODUCT((Inputs!$A$46:$A$85=1)*(Inputs!$D$46:$D$85="boom_local")*(Inputs!$C$46:$C$85&lt;&gt;"boom"))+SUMPRODUCT((Inputs!$A$92:$A$131=1)*(Inputs!$D$92:$D$131="boom_local")*(Inputs!$C$92:$C$131&lt;&gt;"boom"))+SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="boom_local")*(Inputs!$C$138:$C$217&lt;&gt;"boom"))</f>
         <v/>
       </c>
       <c r="D11" s="3">
@@ -45548,16 +45551,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>rope_references</t>
+          <t>node_references</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Segments or hoists referencing a missing or inactive rope</t>
+          <t>References to a missing or inactive node (segment ends, hoist hook/support nodes, hanging nodes' parent)</t>
         </is>
       </c>
       <c r="C12" s="3">
-        <f>SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$B$224:$B$283,Inputs!$A$290:$A$297,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$C$304:$C$311,Inputs!$A$290:$A$297,1)=0))</f>
+        <f>SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$C$224:$C$283,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$D$224:$D$283,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$D$304:$D$311,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(Inputs!$E$304:$E$311&lt;&gt;"")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$E$304:$E$311,Inputs!$A$138:$A$217,1)=0))+SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="hanging")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$I$138:$I$217,Inputs!$A$138:$A$217,1)=0))</f>
         <v/>
       </c>
       <c r="D12" s="3">
@@ -45568,16 +45571,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hoist_without_segments</t>
+          <t>rope_references</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Active hoists whose rope has no active segment</t>
+          <t>Segments or hoists referencing a missing or inactive rope</t>
         </is>
       </c>
       <c r="C13" s="3">
-        <f>SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$224:$B$283,Inputs!$C$304:$C$311,Inputs!$A$224:$A$283,1)=0))</f>
+        <f>SUMPRODUCT((Inputs!$A$224:$A$283=1)*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$B$224:$B$283,Inputs!$A$290:$A$297,1)=0))+SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$290:$B$297,Inputs!$C$304:$C$311,Inputs!$A$290:$A$297,1)=0))</f>
         <v/>
       </c>
       <c r="D13" s="3">
@@ -45588,16 +45591,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>multiple_solve_ropes</t>
+          <t>hoist_without_segments</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Active solve ropes beyond the first (exactly one is allowed)</t>
+          <t>Active hoists whose rope has no active segment</t>
         </is>
       </c>
       <c r="C14" s="3">
-        <f>MAX(0,COUNTIFS(Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"solve")-1)</f>
+        <f>SUMPRODUCT((Inputs!$A$304:$A$311=1)*(COUNTIFS(Inputs!$B$224:$B$283,Inputs!$C$304:$C$311,Inputs!$A$224:$A$283,1)=0))</f>
         <v/>
       </c>
       <c r="D14" s="3">
@@ -45608,16 +45611,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>no_solve_rope</t>
+          <t>multiple_solve_ropes</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1 if no active rope has role solve (the app shows no results then)</t>
+          <t>Active solve ropes beyond the first (exactly one is allowed)</t>
         </is>
       </c>
       <c r="C15" s="3">
-        <f>IF(COUNTIFS(Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"solve")=0,1,0)</f>
+        <f>MAX(0,COUNTIFS(Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"solve")-1)</f>
         <v/>
       </c>
       <c r="D15" s="3">
@@ -45628,16 +45631,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>scene_hoist</t>
+          <t>no_solve_rope</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1 if the scene hoist is not an active hoist with a fixed rope</t>
+          <t>1 if no active rope has role solve (the app shows no results then)</t>
         </is>
       </c>
       <c r="C16" s="3">
-        <f>IF(COUNTIFS(Inputs!$B$304:$B$311,Inputs!$B$26,Inputs!$A$304:$A$311,1)=0,1,IF(COUNTIFS(Inputs!$B$290:$B$297,IFERROR(INDEX(Inputs!$C$304:$C$311,MATCH(Inputs!$B$26&amp;"",Loads!$B$139:$B$146,0)),""),Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"fixed")=0,1,0))</f>
+        <f>IF(COUNTIFS(Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"solve")=0,1,0)</f>
         <v/>
       </c>
       <c r="D16" s="3">
@@ -45648,16 +45651,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>wind_direction</t>
+          <t>scene_hoist</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1 if the scene wind direction is not +X, -X, +Y or -Y</t>
+          <t>1 if the scene hoist is not an active hoist with a fixed rope</t>
         </is>
       </c>
       <c r="C17" s="3">
-        <f>IF(OR(Inputs!$B$33="+X",Inputs!$B$33="-X",Inputs!$B$33="+Y",Inputs!$B$33="-Y"),0,1)</f>
+        <f>IF(COUNTIFS(Inputs!$B$304:$B$311,Inputs!$B$26,Inputs!$A$304:$A$311,1)=0,1,IF(COUNTIFS(Inputs!$B$290:$B$297,IFERROR(INDEX(Inputs!$C$304:$C$311,MATCH(Inputs!$B$26&amp;"",Loads!$B$139:$B$146,0)),""),Inputs!$A$290:$A$297,1,Inputs!$C$290:$C$297,"fixed")=0,1,0))</f>
         <v/>
       </c>
       <c r="D17" s="3">
@@ -45668,16 +45671,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>fixed_nodes_missing</t>
+          <t>wind_direction</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Fixed structure node ids with no active node row</t>
+          <t>1 if the scene wind direction is not +X, -X, +Y or -Y</t>
         </is>
       </c>
       <c r="C18" s="3">
-        <f>COUNTIF($B$36:$B$44,0)</f>
+        <f>IF(OR(Inputs!$B$33="+X",Inputs!$B$33="-X",Inputs!$B$33="+Y",Inputs!$B$33="-Y"),0,1)</f>
         <v/>
       </c>
       <c r="D18" s="3">
@@ -45688,16 +45691,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>hanging_chain</t>
+          <t>fixed_nodes_missing</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Hanging nodes whose parent is itself hanging (only one level is resolved)</t>
+          <t>Fixed structure node ids with no active node row</t>
         </is>
       </c>
       <c r="C19" s="3">
-        <f>SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="hanging")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$I$138:$I$217,Inputs!$D$138:$D$217,"hanging",Inputs!$A$138:$A$217,1)&gt;0))</f>
+        <f>COUNTIF($B$37:$B$45,0)</f>
         <v/>
       </c>
       <c r="D19" s="3">
@@ -45708,16 +45711,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>singular_matrix</t>
+          <t>hanging_chain</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Singular Statics systems (boom 3x3, leg frame 6x6); the boom one is singular without a solve rope</t>
+          <t>Hanging nodes whose parent is itself hanging (only one level is resolved)</t>
         </is>
       </c>
       <c r="C20" s="3">
-        <f>Statics!$B$41+Statics!$B$62</f>
+        <f>SUMPRODUCT((Inputs!$A$138:$A$217=1)*(Inputs!$D$138:$D$217="hanging")*(COUNTIFS(Inputs!$B$138:$B$217,Inputs!$I$138:$I$217,Inputs!$D$138:$D$217,"hanging",Inputs!$A$138:$A$217,1)&gt;0))</f>
         <v/>
       </c>
       <c r="D20" s="3">
@@ -45728,16 +45731,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>zero_boom_width</t>
+          <t>singular_matrix</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1 if the boom width is not &gt; 0 (the app rejects it; the out-of-plane split divides by it, so Results shows a message)</t>
+          <t>Singular Statics systems (boom 3x3, leg frame 6x6); the boom one is singular without a solve rope</t>
         </is>
       </c>
       <c r="C21" s="3">
-        <f>IF(OutOfPlane!$B$20=1,0,1)</f>
+        <f>Statics!$B$41+Statics!$B$62</f>
         <v/>
       </c>
       <c r="D21" s="3">
@@ -45748,16 +45751,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>invalid_bearing_diameter</t>
+          <t>zero_boom_width</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1 if the slewing bearing diameter is typed but not a number &gt; 0 (blank is allowed and hides the bearing line-load rows)</t>
+          <t>1 if the boom width is not &gt; 0 (the app rejects it; the out-of-plane split divides by it, so Results shows a message)</t>
         </is>
       </c>
       <c r="C22" s="3">
-        <f>IF(Inputs!$B$13="",0,IF(ISNUMBER(Inputs!$B$13),IF(Inputs!$B$13&gt;0,0,1),1))</f>
+        <f>IF(OutOfPlane!$B$20=1,0,1)</f>
         <v/>
       </c>
       <c r="D22" s="3">
@@ -45765,66 +45768,67 @@
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>invalid_bearing_diameter</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1 if the slewing bearing diameter is typed but not a number &gt; 0 (blank is allowed and hides the bearing line-load rows)</t>
+        </is>
+      </c>
+      <c r="C23" s="3">
+        <f>IF(Inputs!$B$13="",0,IF(ISNUMBER(Inputs!$B$13),IF(Inputs!$B$13&gt;0,0,1),1))</f>
+        <v/>
+      </c>
+      <c r="D23" s="3">
+        <f>IF(C23=0,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Overflow per table</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Not written</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Typed in guard row</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>mass_points</t>
-        </is>
-      </c>
-      <c r="B27" s="3">
-        <f>Inputs!$G$43</f>
-        <v/>
-      </c>
-      <c r="C27" s="3">
-        <f>COUNTA(Inputs!$A$86:$K$86)</f>
-        <v/>
-      </c>
-      <c r="D27" s="3">
-        <f>B27+C27</f>
-        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>wind_areas</t>
+          <t>mass_points</t>
         </is>
       </c>
       <c r="B28" s="3">
-        <f>Inputs!$G$89</f>
+        <f>Inputs!$G$43</f>
         <v/>
       </c>
       <c r="C28" s="3">
-        <f>COUNTA(Inputs!$A$132:$K$132)</f>
+        <f>COUNTA(Inputs!$A$86:$K$86)</f>
         <v/>
       </c>
       <c r="D28" s="3">
@@ -45835,15 +45839,15 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>nodes</t>
+          <t>wind_areas</t>
         </is>
       </c>
       <c r="B29" s="3">
-        <f>Inputs!$G$135</f>
+        <f>Inputs!$G$89</f>
         <v/>
       </c>
       <c r="C29" s="3">
-        <f>COUNTA(Inputs!$A$218:$K$218)</f>
+        <f>COUNTA(Inputs!$A$132:$K$132)</f>
         <v/>
       </c>
       <c r="D29" s="3">
@@ -45854,15 +45858,15 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>segments</t>
+          <t>nodes</t>
         </is>
       </c>
       <c r="B30" s="3">
-        <f>Inputs!$G$221</f>
+        <f>Inputs!$G$135</f>
         <v/>
       </c>
       <c r="C30" s="3">
-        <f>COUNTA(Inputs!$A$284:$E$284)</f>
+        <f>COUNTA(Inputs!$A$218:$K$218)</f>
         <v/>
       </c>
       <c r="D30" s="3">
@@ -45873,15 +45877,15 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ropes</t>
+          <t>segments</t>
         </is>
       </c>
       <c r="B31" s="3">
-        <f>Inputs!$G$287</f>
+        <f>Inputs!$G$221</f>
         <v/>
       </c>
       <c r="C31" s="3">
-        <f>COUNTA(Inputs!$A$298:$C$298)</f>
+        <f>COUNTA(Inputs!$A$284:$E$284)</f>
         <v/>
       </c>
       <c r="D31" s="3">
@@ -45892,15 +45896,15 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>hoists</t>
+          <t>ropes</t>
         </is>
       </c>
       <c r="B32" s="3">
-        <f>Inputs!$G$301</f>
+        <f>Inputs!$G$287</f>
         <v/>
       </c>
       <c r="C32" s="3">
-        <f>COUNTA(Inputs!$A$312:$Q$312)</f>
+        <f>COUNTA(Inputs!$A$298:$C$298)</f>
         <v/>
       </c>
       <c r="D32" s="3">
@@ -45908,28 +45912,36 @@
         <v/>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>hoists</t>
+        </is>
+      </c>
+      <c r="B33" s="3">
+        <f>Inputs!$G$301</f>
+        <v/>
+      </c>
+      <c r="C33" s="3">
+        <f>COUNTA(Inputs!$A$312:$Q$312)</f>
+        <v/>
+      </c>
+      <c r="D33" s="3">
+        <f>B33+C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Fixed structure nodes (active rows with this id)</t>
         </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>boom_heel</t>
-        </is>
-      </c>
-      <c r="B36" s="3">
-        <f>COUNTIFS(Inputs!$B$138:$B$217,A36,Inputs!$A$138:$A$217,1)</f>
-        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>platform_heel</t>
+          <t>boom_heel</t>
         </is>
       </c>
       <c r="B37" s="3">
@@ -45940,7 +45952,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>rear_top</t>
+          <t>platform_heel</t>
         </is>
       </c>
       <c r="B38" s="3">
@@ -45951,7 +45963,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>front_top</t>
+          <t>rear_top</t>
         </is>
       </c>
       <c r="B39" s="3">
@@ -45962,7 +45974,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>rear_base</t>
+          <t>front_top</t>
         </is>
       </c>
       <c r="B40" s="3">
@@ -45973,7 +45985,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>platform_rear</t>
+          <t>rear_base</t>
         </is>
       </c>
       <c r="B41" s="3">
@@ -45984,7 +45996,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>front_base</t>
+          <t>platform_rear</t>
         </is>
       </c>
       <c r="B42" s="3">
@@ -45995,7 +46007,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>platform_front</t>
+          <t>front_base</t>
         </is>
       </c>
       <c r="B43" s="3">
@@ -46006,7 +46018,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>platform_base</t>
+          <t>platform_front</t>
         </is>
       </c>
       <c r="B44" s="3">
@@ -46014,8 +46026,19 @@
         <v/>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>platform_base</t>
+        </is>
+      </c>
+      <c r="B45" s="3">
+        <f>COUNTIFS(Inputs!$B$138:$B$217,A45,Inputs!$A$138:$A$217,1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C6:C22">
+  <conditionalFormatting sqref="C6:C23">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>